<commit_message>
feat(executive): elevate workbook to 5 C-Level sheets with ROI simulator and generate official walkthrough Word guide
</commit_message>
<xml_diff>
--- a/tiktok_performance_analysis.xlsx
+++ b/tiktok_performance_analysis.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Creators &amp; Treemap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Deep Dive &amp; Factors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Clean Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators &amp; Treemap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deep Dive &amp; Factors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Simulator &amp; ROI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Data" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0 €"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0 M"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,7 +38,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -53,7 +56,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000D9488"/>
-      <sz val="18"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -65,19 +68,19 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
-      <sz val="18"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00D97706"/>
-      <sz val="18"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00BE185D"/>
-      <sz val="18"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -102,8 +105,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="17"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -167,6 +176,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
+        <bgColor rgb="00B45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00334155"/>
         <bgColor rgb="00334155"/>
       </patternFill>
@@ -198,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -275,7 +315,41 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -355,7 +429,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -370,13 +444,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -385,7 +459,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -400,13 +474,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -425,13 +499,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -440,7 +514,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -455,13 +529,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2866,6 +2940,532 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:K27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SIMULATEUR BUDGÉTAIRE &amp; PROJECTIONS DE PERFORMANCE (CAMPAGNE B2C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Modélisation financière sur une enveloppe type de 100 000 € : Comparatif Scénario Classique vs Recommandation Data-Driven</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>BUDGET ALLOUÉ SIMULATION</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PORTÉE ESTIMÉE DATA-DRIVEN</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>CPM ESTIMÉ DATA-DRIVEN</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>ENGAGEMENT MOYEN ATTENDU</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="36" t="inlineStr">
+        <is>
+          <t>100 000 €</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>118,5 M</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>0,84 €</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>18,6 %</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Enveloppe nette influenceurs</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>+114% vs Scénario Classique</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Coût pour 1 000 vues divisé par 2</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>Fidélisation communautaire forte</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>1. COMPARAISON STRATÉGIQUE DES DEUX SCÉNARIOS D'INVESTISSEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Indicateur Clé</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Scénario A : Approche Classique (100% Mega)</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>Scénario B : Approche Data-Driven (70% Micro/Mid + 30% Mega)</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Différentiel Performance</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>Impact Business pour la Marque B2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>Nombre de Créateurs Activés</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>2 créateurs Mega</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>14 créateurs (11 Micro/Mid + 3 Mega)</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>+600% de partenaires</t>
+        </is>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>Diversification maximale du risque algorithmique</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>Budget Consacré</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>100 000 € (2 x 50k€)</t>
+        </is>
+      </c>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>100 000 € (70k€ Micro/Mid + 30k€ Mega)</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Enveloppe identique</t>
+        </is>
+      </c>
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>Optimisation de l'allocation sans surcoût</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>Vues Totales Estimées</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>55,2 M de vues</t>
+        </is>
+      </c>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>118,5 M de vues</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>+114% de portée (+63,3M)</t>
+        </is>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>Audience doublée grâce au sur-rendement des micro-comptes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Taux d'Engagement Projeté</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>14,2 % (Interactions / Vues)</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>18,6 % (Interactions / Vues)</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>+4,4 pts d'engagement</t>
+        </is>
+      </c>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>Meilleure conversion organique et bouche-à-oreille</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>Total Interactions Projeté</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>7,84 Millions de likes/comm/part</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>22,04 Millions de likes/comm/part</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>+181% d'interactions</t>
+        </is>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>Génération de contenu utilisateur et partage viral massif</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Coût pour 1 000 Vues (CPM)</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>1,81 € par 1 000 vues</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>0,84 € par 1 000 vues</t>
+        </is>
+      </c>
+      <c r="E17" s="41" t="inlineStr">
+        <is>
+          <t>-54% sur le coût par vue</t>
+        </is>
+      </c>
+      <c r="F17" s="39" t="inlineStr">
+        <is>
+          <t>Division par deux du coût d'acquisition de visibilité</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>Vulnérabilité Algorithmique</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>Extrême (si 1 vidéo 'flop', 50% du budget est perdu)</t>
+        </is>
+      </c>
+      <c r="D18" s="40" t="inlineStr">
+        <is>
+          <t>Très faible (panier diversifié de 14 vidéos indépendantes)</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>Sécurité renforcée</t>
+        </is>
+      </c>
+      <c r="F18" s="39" t="inlineStr">
+        <is>
+          <t>Garantie de résultat statistique pour la marque</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>2. MODÉLISATION DU PANIER DE CASTING RECOMMANDÉ (MIX 70 / 30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Segment Créateur</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Budget Moyen / Créateur</t>
+        </is>
+      </c>
+      <c r="E23" s="42" t="inlineStr">
+        <is>
+          <t>Budget Total Segment</t>
+        </is>
+      </c>
+      <c r="F23" s="42" t="inlineStr">
+        <is>
+          <t>Vues Moyennes / Créateur</t>
+        </is>
+      </c>
+      <c r="G23" s="42" t="inlineStr">
+        <is>
+          <t>Total Vues Segment (M)</t>
+        </is>
+      </c>
+      <c r="H23" s="42" t="inlineStr">
+        <is>
+          <t>Taux Engagement Moyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>Micro/Nano (&lt; 1M followers)</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="44" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E24" s="44" t="n">
+        <v>28000</v>
+      </c>
+      <c r="F24" s="45" t="n">
+        <v>50800000</v>
+      </c>
+      <c r="G24" s="46">
+        <f>D24*E24/1000000</f>
+        <v/>
+      </c>
+      <c r="H24" s="43" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>Mid/Macro (1M - 5M followers)</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="44" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E25" s="44" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F25" s="45" t="n">
+        <v>82600000</v>
+      </c>
+      <c r="G25" s="46">
+        <f>D25*E25/1000000</f>
+        <v/>
+      </c>
+      <c r="H25" s="43" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>Mega Influenceurs (5M+ followers)</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="44" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E26" s="44" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F26" s="45" t="n">
+        <v>68700000</v>
+      </c>
+      <c r="G26" s="46">
+        <f>D26*E26/1000000</f>
+        <v/>
+      </c>
+      <c r="H26" s="43" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="47" t="inlineStr">
+        <is>
+          <t>TOTAL CAMPAGNE</t>
+        </is>
+      </c>
+      <c r="C27" s="48">
+        <f>SUM(C24:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" s="50">
+        <f>SUM(E24:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="51">
+        <f>SUM(G24:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="48" t="inlineStr">
+        <is>
+          <t>18.6% (Moy. pondérée)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B3:K3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2888,14 +3488,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t xml:space="preserve">  BASE DE DONNÉES PRÉPARÉE &amp; NETTOYÉE (100 OBSERVATIONS) — FORMAT CLIENT</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  Conformité RGPD &amp; Règles Agence : Anonymisation des PII, suppression des identifiants techniques opaques et des données privées.</t>
         </is>
@@ -2903,82 +3503,82 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="54" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="54" t="inlineStr">
         <is>
           <t>Handle_Createur</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="54" t="inlineStr">
         <is>
           <t>Nom_Affiche</t>
         </is>
       </c>
-      <c r="D4" s="36" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
       </c>
-      <c r="E4" s="36" t="inlineStr">
+      <c r="E4" s="54" t="inlineStr">
         <is>
           <t>Segment_Followers</t>
         </is>
       </c>
-      <c r="F4" s="36" t="inlineStr">
+      <c r="F4" s="54" t="inlineStr">
         <is>
           <t>Abonnés</t>
         </is>
       </c>
-      <c r="G4" s="36" t="inlineStr">
+      <c r="G4" s="54" t="inlineStr">
         <is>
           <t>Duree_Sec</t>
         </is>
       </c>
-      <c r="H4" s="36" t="inlineStr">
+      <c r="H4" s="54" t="inlineStr">
         <is>
           <t>Vues</t>
         </is>
       </c>
-      <c r="I4" s="36" t="inlineStr">
+      <c r="I4" s="54" t="inlineStr">
         <is>
           <t>Likes</t>
         </is>
       </c>
-      <c r="J4" s="36" t="inlineStr">
+      <c r="J4" s="54" t="inlineStr">
         <is>
           <t>Commentaires</t>
         </is>
       </c>
-      <c r="K4" s="36" t="inlineStr">
+      <c r="K4" s="54" t="inlineStr">
         <is>
           <t>Partages</t>
         </is>
       </c>
-      <c r="L4" s="36" t="inlineStr">
+      <c r="L4" s="54" t="inlineStr">
         <is>
           <t>Total_Interactions</t>
         </is>
       </c>
-      <c r="M4" s="36" t="inlineStr">
+      <c r="M4" s="54" t="inlineStr">
         <is>
           <t>Taux_Engagement</t>
         </is>
       </c>
-      <c r="N4" s="36" t="inlineStr">
+      <c r="N4" s="54" t="inlineStr">
         <is>
           <t>Multiplicateur_Viral</t>
         </is>
       </c>
-      <c r="O4" s="36" t="inlineStr">
+      <c r="O4" s="54" t="inlineStr">
         <is>
           <t>Audio_Original</t>
         </is>
       </c>
-      <c r="P4" s="36" t="inlineStr">
+      <c r="P4" s="54" t="inlineStr">
         <is>
           <t>Badge_Certifie</t>
         </is>

</xml_diff>